<commit_message>
feat: Add study opt-in/out functionality and admin access management
- Implemented the study opt-in/out feature in a new `studyopt.js` file, allowing users to select their participation status for various studies.
- Introduced a new function `loadOptInOutTable` to dynamically load and display the opt-in/out selections based on user email.
- Enhanced CSV parsing in `shared.js` to handle quoted values correctly in the `csv2Json` function.
- Added `extractRequestedConsortia` function to extract requested consortia/study data from text.
- Updated the `loadStudyAccessAdminTable` function to manage admin access and display requested studies with user details.
</commit_message>
<xml_diff>
--- a/src/data/DataPlatform-Out-in-out.xlsx
+++ b/src/data/DataPlatform-Out-in-out.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahearntu\AppData\Local\Box\Box for Office\6954560291\Temp\ppcjkjyl.ppz\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kopchickbp\Documents\DCEG_Data_Platforms\confluence\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3E1F082-FA5E-4519-A8DD-3DD19A244E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D66F7C-B2E4-4B02-BC47-ED8A21509956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{350D2FCD-1D3B-4D9D-B201-6339E00B3D2C}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{350D2FCD-1D3B-4D9D-B201-6339E00B3D2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
   <si>
     <t>Name</t>
   </si>
@@ -327,16 +327,48 @@
   </si>
   <si>
     <t>EDSMAR</t>
+  </si>
+  <si>
+    <t>Ben Kopchick</t>
+  </si>
+  <si>
+    <t>kopchickbp@nih.gov</t>
+  </si>
+  <si>
+    <t>Test Study 1</t>
+  </si>
+  <si>
+    <t>ST1</t>
+  </si>
+  <si>
+    <t>Test Study 2</t>
+  </si>
+  <si>
+    <t>TS2</t>
+  </si>
+  <si>
+    <t>Test Study 3</t>
+  </si>
+  <si>
+    <t>TS3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -359,20 +391,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1271,20 +1305,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1072664F-2A48-4061-8ACE-ED4424A887C9}">
-  <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="103.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="103.7109375" customWidth="1"/>
-    <col min="5" max="5" width="72.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="46.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="103.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="103.7265625" customWidth="1"/>
+    <col min="5" max="5" width="72.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="46.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1310,7 +1344,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1325,11 +1359,11 @@
         <v>BRISBANE</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>23</v>
       </c>
       <c r="C3" t="s">
@@ -1340,7 +1374,7 @@
         <v>ROCS</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>48</v>
       </c>
@@ -1354,20 +1388,20 @@
         <f>VLOOKUP(C4,[1]Sheet1!$A$2:$F$30,6,FALSE)</f>
         <v>SHARE</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>81</v>
       </c>
       <c r="F4" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>83</v>
       </c>
       <c r="H4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -1381,14 +1415,14 @@
         <f>VLOOKUP(C5,[1]Sheet1!$A$2:$F$30,6,FALSE)</f>
         <v>SACGEN-B</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F5" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1403,7 +1437,7 @@
         <v>ABRECANE</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1417,7 +1451,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -1432,7 +1466,7 @@
         <v>ARSENIC</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>45</v>
       </c>
@@ -1447,7 +1481,7 @@
         <v>CAMACOL</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>58</v>
       </c>
@@ -1462,7 +1496,7 @@
         <v>Komen</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -1476,7 +1510,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1491,7 +1525,7 @@
         <v xml:space="preserve">CanPath </v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>63</v>
       </c>
@@ -1505,7 +1539,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>66</v>
       </c>
@@ -1520,7 +1554,7 @@
         <v>UPENN_HighRIsk</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -1535,7 +1569,7 @@
         <v>Pathways</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>75</v>
       </c>
@@ -1550,7 +1584,7 @@
         <v>ICSBCS</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>61</v>
       </c>
@@ -1565,7 +1599,7 @@
         <v>Komen</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -1580,7 +1614,7 @@
         <v>PAK_BCCC</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1595,7 +1629,7 @@
         <v>IndianBCRP</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>52</v>
       </c>
@@ -1609,20 +1643,20 @@
         <f>VLOOKUP(C20,[1]Sheet1!$A$2:$F$30,6,FALSE)</f>
         <v>SABC</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="2" t="s">
         <v>90</v>
       </c>
       <c r="F20" t="s">
         <v>91</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H20" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -1637,7 +1671,7 @@
         <v>LACAM</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -1652,7 +1686,7 @@
         <v>BRISBANE</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>69</v>
       </c>
@@ -1667,7 +1701,7 @@
         <v>UPENN_HighRIsk</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>71</v>
       </c>
@@ -1682,7 +1716,7 @@
         <v>WISE</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -1697,7 +1731,7 @@
         <v>ABC-DO</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -1709,6 +1743,32 @@
       </c>
       <c r="D26" t="s">
         <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C27" t="s">
+        <v>96</v>
+      </c>
+      <c r="D27" t="s">
+        <v>97</v>
+      </c>
+      <c r="E27" t="s">
+        <v>98</v>
+      </c>
+      <c r="F27" t="s">
+        <v>99</v>
+      </c>
+      <c r="G27" t="s">
+        <v>100</v>
+      </c>
+      <c r="H27" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1717,6 +1777,9 @@
       <sortCondition ref="A1:A26"/>
     </sortState>
   </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="B27" r:id="rId1" xr:uid="{3B97577C-AFDE-4D69-B344-83DB1C69D070}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: Update DataPlatform-Out-in-out.xlsx with new data
</commit_message>
<xml_diff>
--- a/src/data/DataPlatform-Out-in-out.xlsx
+++ b/src/data/DataPlatform-Out-in-out.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kopchickbp\Documents\DCEG_Data_Platforms\confluence\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D66F7C-B2E4-4B02-BC47-ED8A21509956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED500A3-74B0-4CA2-9EC2-D1D8BC26267D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{350D2FCD-1D3B-4D9D-B201-6339E00B3D2C}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{350D2FCD-1D3B-4D9D-B201-6339E00B3D2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="107">
   <si>
     <t>Name</t>
   </si>
@@ -351,13 +351,28 @@
   </si>
   <si>
     <t>TS3</t>
+  </si>
+  <si>
+    <t>Thomas Ahearn</t>
+  </si>
+  <si>
+    <t>ahearntu@nih.gov</t>
+  </si>
+  <si>
+    <t>ST2</t>
+  </si>
+  <si>
+    <t>Test Study 4</t>
+  </si>
+  <si>
+    <t>TS4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -369,6 +384,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1305,7 +1326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1072664F-2A48-4061-8ACE-ED4424A887C9}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.54296875" bestFit="1" customWidth="1"/>
@@ -1771,12 +1792,39 @@
         <v>101</v>
       </c>
     </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" t="s">
+        <v>104</v>
+      </c>
+      <c r="E28" t="s">
+        <v>100</v>
+      </c>
+      <c r="F28" t="s">
+        <v>101</v>
+      </c>
+      <c r="G28" t="s">
+        <v>105</v>
+      </c>
+      <c r="H28" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C26" xr:uid="{1072664F-2A48-4061-8ACE-ED4424A887C9}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C26">
       <sortCondition ref="A1:A26"/>
     </sortState>
   </autoFilter>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B27" r:id="rId1" xr:uid="{3B97577C-AFDE-4D69-B344-83DB1C69D070}"/>
   </hyperlinks>

</xml_diff>